<commit_message>
Checkpoint 7 weeks of engine work: move-signature channel, QA gates, demo build
Brings origin up to date after 50 days of local-only development.

Engine:
- rhetorical move-signature novelty channel (fingerprints, config vocabulary)
- seed classification and genre-saturation steering
- similarity screen and qa_checks gates
- topic-shape and render-stance component families
- multi-provider stage pins with never-fatal fallback

Tooling and surfaces:
- tests/ (163 cases) — never previously committed
- tools/build_demo_snapshot.py and the static demo/ walkthrough
- .github/workflows/deploy-demo.yml with a cost-leak build guard
- GUI remote launcher and provider key-provenance reporting

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RC_Tracker_new.xlsx
+++ b/RC_Tracker_new.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2528,6 +2528,450 @@
       <c r="G58" t="inlineStr">
         <is>
           <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RC-ELITE-260726-0032</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>RC_ELITE_260822_02</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Pipeline approved (score 8.6); passed duplicate check, word count 527 (elite band), length-bias clean (0/6 longest); placed into Week_5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0019</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>RC_HARD_260815_05</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Week_4_15_08</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Was needs_review, user approved 2026-07-26; passed duplicate check, word count 545 (45 over hard band, flagged), length-bias clean (2/6 longest -- Q2,Q6 -- thesis Q1 not longest); placed into Week_4 (completed to 5/5)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0021</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>RC_HARD_260822_01</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Was needs_review, user approved 2026-07-26; passed duplicate check, word count 556 (56 over hard band, flagged), length-bias clean (0/6 longest); placed into new Week_5 Hard slot</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0015</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>RC_HARD_260822_02</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Was needs_review with verdict "skipped_budget" (judge never ran, not a quality rejection); manually judged 2026-07-26 by same 5-category rubric -- family_realization 8, ending_behavior 9, voice_consistency 8, distractor_efficiency 8, explanation_quality 8, average 8.2, verdict approve; db updated to approved/8.2; passed duplicate check (no match anywhere in shipped corpus), word count 501 (hard band), length-bias clean (0/6 longest, thesis not longest); placed into Week_5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>RC-ELITE-260707-0022</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>RC_ELITE_260822_03</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Was needs_review; manually judged 2026-07-26 (family_realization 9, ending_behavior 8, voice_consistency 9, distractor_efficiency 9, explanation_quality 9, avg 8.8, corroborates pipeline judge) -- approve. Original had length-bias FAIL (4/6 longest: Q2,Q3,Q4,Q5); manually fixed by trimming those 4 option wordings (no meaning change) -- re-verified 0/6 flags, thesis not longest. Word count 575 (25 over elite band, within tolerance). Passed duplicate check.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>RC-ELITE-260711-0023</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>RC_ELITE_260822_04</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Was rejected_novelty (verdict not_run_novelty, flagged nearest to RC-ELITE-260706-0005 and RC_E_0706_1); manually judged 2026-07-26 (avg 7.8) -- approve. Manually compared against both flagged neighbors: topics and core mechanisms differ substantively (evidence-scope-limitation vs incommensurable-values vs mutual-blindness-of-two-accounts) -- NOT a near-duplicate, cleared to ship. Original had length-bias FAIL (3/6 longest: Q2,Q3,Q5); manually fixed by trimming those 3 option wordings -- re-verified 0/6 flags, thesis not longest. Word count 532 (in band). Passed duplicate check.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>RC-ELITE-260711-0024</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>RC_ELITE_260822_05</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Was needs_review; manually judged 2026-07-26 (avg 8.4, corroborates pipeline judge) -- approve. Original had length-bias FAIL (3/6 longest: Q4,Q5,Q6) AND word count 414 (86 under elite band); manually fixed by expanding paragraphs 2 and 3 with additional concrete detail (no argument change) to reach word count 505, and trimming Q4/Q5/Q6 option wordings -- re-verified 0/6 flags, thesis not longest, word count now in band. Passed duplicate check.</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0022</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>RC_HARD_260822_03</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Pipeline approved (score 8.6); passed duplicate check, word count 518 (18 over hard band, within tolerance), length-bias clean (0/6 longest); placed into Week_5</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0023</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>RC_HARD_260822_04</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Pipeline approved (score 8.0); passed duplicate check, word count 536 (36 over hard band, flagged), length-bias clean (1/6, Q5, thesis not longest); placed into Week_5</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0024</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>RC_HARD_260822_05</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Pipeline approved (score 8.6); passed duplicate check, word count 524 (24 over hard band, flagged), length-bias clean (1/6, Q4, thesis not longest); placed into Week_5 (completed to 5/5)</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>RC-HARD-260726-0025</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>RC_HARD_260829_01</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Week_6_29_08</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Was needs_review; manually judged 2026-07-26 (family_realization 9, ending_behavior 9, voice_consistency 8, distractor_efficiency 8, explanation_quality 8, avg 8.4) -- approve; db updated to approved/8.4. Passed duplicate check, word count 548 (48 over hard band, flagged), length-bias clean (0/6 longest); placed into new Week_6</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>RC-MEDIUM-260726-0021</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>RC_MEDIUM_260822_02</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Week_5_22_08</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Pipeline approved (score 8.8, verdict approve, verified via judge_json before shipping); passed duplicate check, word count 503 (53 over medium band 400-450, flagged), length-bias clean (0/6 longest, thesis not longest); placed into Week_5 (completed to 2/2 -- Week_5 now full across all three tiers)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
         </is>
       </c>
     </row>

</xml_diff>